<commit_message>
Capturing next level of functionality. Initial tetsting of the French data files complete. Need to add some organization, the commanders should be at the top of the list when we can.
</commit_message>
<xml_diff>
--- a/assets/ESR Formations-Austria.xlsx
+++ b/assets/ESR Formations-Austria.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR_NewRecruit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR_NewRecruit/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{2659956D-E850-43CB-8414-2D912463ECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8F3225E-10E3-43A3-BEC0-1E0F9F25DA5D}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="8_{2659956D-E850-43CB-8414-2D912463ECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ADAC048-A92A-427D-BCF7-F03096455E1A}"/>
   <bookViews>
-    <workbookView xWindow="4455" yWindow="90" windowWidth="28275" windowHeight="14700" activeTab="1" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
+    <workbookView xWindow="1050" yWindow="0" windowWidth="26610" windowHeight="14700" activeTab="1" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
   </bookViews>
   <sheets>
     <sheet name="BaselineFormations" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="57">
   <si>
     <t>Formation</t>
   </si>
@@ -354,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -371,29 +371,26 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -736,7 +733,7 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="25.5703125" style="13" customWidth="1"/>
+    <col min="1" max="10" width="25.5703125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -758,23 +755,21 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -783,60 +778,54 @@
       <c r="E2" s="3">
         <v>4</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
+      <c r="F2" s="11"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" spans="1:10" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="3">
         <v>4</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="10" t="s">
+      <c r="F3" s="11"/>
+      <c r="I3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="8" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="10" t="s">
+      <c r="F4" s="11"/>
+      <c r="I4" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="12" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -845,33 +834,29 @@
       <c r="E5" s="5">
         <v>9</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="10" t="s">
+      <c r="F5" s="12"/>
+      <c r="I5" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="8" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
       <c r="D6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="5">
         <v>1</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="10" t="s">
+      <c r="F6" s="12"/>
+      <c r="I6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="8" t="s">
         <v>38</v>
       </c>
     </row>
@@ -892,12 +877,10 @@
         <v>12</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="8" t="s">
         <v>38</v>
       </c>
     </row>
@@ -918,89 +901,81 @@
         <v>8</v>
       </c>
       <c r="F8" s="4"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="11"/>
-      <c r="F9" s="6" t="s">
+      <c r="E9" s="9"/>
+      <c r="F9" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="10" t="s">
+      <c r="F10" s="11"/>
+      <c r="I10" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="10" t="s">
+      <c r="F11" s="11"/>
+      <c r="I11" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="12" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -1009,44 +984,40 @@
       <c r="E12" s="5">
         <v>6</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="10" t="s">
+      <c r="F12" s="12"/>
+      <c r="I12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
       <c r="D13" s="4" t="s">
         <v>28</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="10" t="s">
+      <c r="F13" s="12"/>
+      <c r="I13" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
@@ -1055,77 +1026,63 @@
       <c r="E14" s="3">
         <v>2</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="10" t="s">
+      <c r="F14" s="11"/>
+      <c r="I14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J14" s="10" t="s">
+      <c r="J14" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E15" s="3">
         <v>3</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="10" t="s">
+      <c r="F15" s="11"/>
+      <c r="I15" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J15" s="10" t="s">
+      <c r="J15" s="8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="3">
         <v>2</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="10" t="s">
+      <c r="F16" s="11"/>
+      <c r="I16" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="J16" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="10" t="s">
+    <row r="17" spans="9:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I17" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I18" s="10" t="s">
+    <row r="18" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I18" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="J18" s="8" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1165,69 +1122,69 @@
     <col min="4" max="18" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:19" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="str" cm="1">
+      <c r="D1" s="10" t="str" cm="1">
         <f t="array" ref="D1:S1">TRANSPOSE( BaselineFormations!I3:I18 )</f>
         <v>Grenzer</v>
       </c>
-      <c r="E1" s="13" t="str">
+      <c r="E1" s="10" t="str">
         <v>Jägere</v>
       </c>
-      <c r="F1" s="13" t="str">
+      <c r="F1" s="10" t="str">
         <v>Infanterie</v>
       </c>
-      <c r="G1" s="13" t="str">
+      <c r="G1" s="10" t="str">
         <v>Grenadiere</v>
       </c>
-      <c r="H1" s="13" t="str">
+      <c r="H1" s="10" t="str">
         <v>Landwehr</v>
       </c>
-      <c r="I1" s="13" t="str">
+      <c r="I1" s="10" t="str">
         <v>Pioneere</v>
       </c>
-      <c r="J1" s="13" t="str">
+      <c r="J1" s="10" t="str">
         <v>Sapeurs</v>
       </c>
-      <c r="K1" s="13" t="str">
+      <c r="K1" s="10" t="str">
         <v>Kürassiere</v>
       </c>
-      <c r="L1" s="13" t="str">
+      <c r="L1" s="10" t="str">
         <v>Chevaulegers</v>
       </c>
-      <c r="M1" s="13" t="str">
+      <c r="M1" s="10" t="str">
         <v>Dragoner</v>
       </c>
-      <c r="N1" s="13" t="str">
+      <c r="N1" s="10" t="str">
         <v>Husaren</v>
       </c>
-      <c r="O1" s="13" t="str">
+      <c r="O1" s="10" t="str">
         <v>Ulanen</v>
       </c>
-      <c r="P1" s="13" t="str">
+      <c r="P1" s="10" t="str">
         <v>Position-Batterien</v>
       </c>
-      <c r="Q1" s="13" t="str">
+      <c r="Q1" s="10" t="str">
         <v>Brigade-Batterien</v>
       </c>
-      <c r="R1" s="13" t="str">
+      <c r="R1" s="10" t="str">
         <v>Leitche Artillerie</v>
       </c>
-      <c r="S1" s="13" t="str">
+      <c r="S1" s="10" t="str">
         <v>Würst Artillerie</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:C8">_xlfn._xlws.FILTER(BaselineFormations!A:C,(BaselineFormations!A:A&lt;&gt;"Formation")*(NOT(ISBLANK(BaselineFormations!A:A))))</f>
+        <f t="array" ref="A2:C8">_xlfn.LET(_xlpm.data,_xlfn._xlws.FILTER(BaselineFormations!A:C,(BaselineFormations!A:A&lt;&gt;"Formation")*(NOT(ISBLANK(BaselineFormations!A:A)))),IF(_xlpm.data=0,"",_xlpm.data))</f>
         <v>Avant Garde</v>
       </c>
       <c r="B2" t="str">
@@ -1243,6 +1200,12 @@
         <v>54</v>
       </c>
       <c r="L2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>54</v>
+      </c>
+      <c r="R2" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1278,6 +1241,9 @@
         <v>54</v>
       </c>
       <c r="Q3" t="s">
+        <v>54</v>
+      </c>
+      <c r="R3" t="s">
         <v>54</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Completed entry for the Mixed formations, completed Allied formation. All inside of the Formations.cat file. Tested with Wurttemberg.
</commit_message>
<xml_diff>
--- a/assets/ESR Formations-Austria.xlsx
+++ b/assets/ESR Formations-Austria.xlsx
@@ -5,20 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR_NewRecruit/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="136" documentId="8_{2659956D-E850-43CB-8414-2D912463ECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E77A4009-BF4C-4E8B-B813-1DA2A9D22C00}"/>
+  <xr:revisionPtr revIDLastSave="156" documentId="8_{2659956D-E850-43CB-8414-2D912463ECF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{883D82D0-0355-4550-AD9E-67207041195E}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="375" windowWidth="26610" windowHeight="14595" activeTab="1" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
+    <workbookView xWindow="750" yWindow="600" windowWidth="26610" windowHeight="14595" activeTab="1" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
   </bookViews>
   <sheets>
     <sheet name="BaselineFormations" sheetId="1" r:id="rId1"/>
     <sheet name="ExpandedFormations" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="FromArray_1">_xlfn.ANCHORARRAY(ExpandedFormations!$A$2)</definedName>
-    <definedName name="FromArray_3">_xlfn.ANCHORARRAY(ExpandedFormations!$D$2)</definedName>
+    <definedName name="FromArray_1">_xlfn.ANCHORARRAY(ExpandedFormations!$A$3)</definedName>
+    <definedName name="FromArray_3">_xlfn.ANCHORARRAY(ExpandedFormations!$D$3)</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="60">
   <si>
     <t>Formation</t>
   </si>
@@ -254,6 +254,9 @@
   </si>
   <si>
     <t>AU Würst Artillerie</t>
+  </si>
+  <si>
+    <t>AU Mixed</t>
   </si>
 </sst>
 </file>
@@ -413,10 +416,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1094,18 +1093,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="C12:C13"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:C4"/>
@@ -1114,6 +1101,18 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="F5:F6"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="F12:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1121,7 +1120,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A52F401-E5BC-41DA-8596-65382229DEB1}">
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="24.85546875" customWidth="1"/>
@@ -1188,65 +1187,80 @@
         <v>AU Würst Artillerie</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:C8">_xlfn.LET(_xlpm.data,_xlfn._xlws.FILTER(BaselineFormations!A:C,(BaselineFormations!A:A&lt;&gt;"Formation")*(NOT(ISBLANK(BaselineFormations!A:A)))),IF(_xlpm.data=0,"",_xlpm.data))</f>
+    <row r="2" spans="1:19" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="str" cm="1">
+        <f t="array" ref="A3:C9">_xlfn.LET(_xlpm.data,_xlfn._xlws.FILTER(BaselineFormations!A:C,(BaselineFormations!A:A&lt;&gt;"Formation")*(NOT(ISBLANK(BaselineFormations!A:A)))),IF(_xlpm.data=0,"",_xlpm.data))</f>
         <v>AU Avant Garde</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
         <v>Mixed</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C3" t="str">
         <v>Rapid Deployment</v>
       </c>
-      <c r="D2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" t="s">
-        <v>35</v>
-      </c>
-      <c r="L2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>35</v>
-      </c>
-      <c r="R2" t="s">
-        <v>35</v>
-      </c>
-      <c r="S2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="str">
-        <v>AU Infanterie Division</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Infantry</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Big Battalions*</v>
+      <c r="D3" t="s">
+        <v>35</v>
       </c>
       <c r="E3" t="s">
         <v>35</v>
       </c>
-      <c r="F3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" t="s">
-        <v>35</v>
-      </c>
-      <c r="P3" t="s">
+      <c r="L3" t="s">
         <v>35</v>
       </c>
       <c r="Q3" t="s">
@@ -1261,27 +1275,27 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
-        <v>AU Reservieren Division</v>
+        <v>AU Infanterie Division</v>
       </c>
       <c r="B4" t="str">
         <v>Infantry</v>
       </c>
       <c r="C4" t="str">
-        <v>Enthusiastic</v>
-      </c>
-      <c r="G4" t="s">
+        <v>Big Battalions*</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
         <v>35</v>
       </c>
       <c r="I4" t="s">
         <v>35</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" t="s">
         <v>35</v>
       </c>
       <c r="O4" t="s">
@@ -1302,13 +1316,22 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <v>AU Leichte Kavallerie Brigade</v>
+        <v>AU Reservieren Division</v>
       </c>
       <c r="B5" t="str">
-        <v>Cavalry</v>
+        <v>Infantry</v>
       </c>
       <c r="C5" t="str">
-        <v>Rapid Deployment</v>
+        <v>Enthusiastic</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
       </c>
       <c r="L5" t="s">
         <v>35</v>
@@ -1317,6 +1340,15 @@
         <v>35</v>
       </c>
       <c r="O5" t="s">
+        <v>35</v>
+      </c>
+      <c r="P5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R5" t="s">
         <v>35</v>
       </c>
       <c r="S5" t="s">
@@ -1325,7 +1357,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>AU Kavallerie Brigade/Division</v>
+        <v>AU Leichte Kavallerie Brigade</v>
       </c>
       <c r="B6" t="str">
         <v>Cavalry</v>
@@ -1336,7 +1368,10 @@
       <c r="L6" t="s">
         <v>35</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" t="s">
         <v>35</v>
       </c>
       <c r="S6" t="s">
@@ -1345,7 +1380,7 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <v>AU Kürassier Division</v>
+        <v>AU Kavallerie Brigade/Division</v>
       </c>
       <c r="B7" t="str">
         <v>Cavalry</v>
@@ -1353,7 +1388,10 @@
       <c r="C7" t="str">
         <v>Rapid Deployment</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" t="s">
         <v>35</v>
       </c>
       <c r="S7" t="s">
@@ -1362,30 +1400,47 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
+        <v>AU Kürassier Division</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Cavalry</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Rapid Deployment</v>
+      </c>
+      <c r="K8" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
         <v>AU Korps Reservieren</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v>Artillery</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C9" t="str">
         <v>Reinforcements</v>
       </c>
-      <c r="I8" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" t="s">
-        <v>35</v>
-      </c>
-      <c r="P8" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>35</v>
-      </c>
-      <c r="R8" t="s">
-        <v>35</v>
-      </c>
-      <c r="S8" t="s">
+      <c r="I9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" t="s">
+        <v>35</v>
+      </c>
+      <c r="P9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>35</v>
+      </c>
+      <c r="R9" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>